<commit_message>
changes to config for input
</commit_message>
<xml_diff>
--- a/OrderbookAutomation/output/Business_Master_Data.xlsx
+++ b/OrderbookAutomation/output/Business_Master_Data.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Statistics" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master_Data'!$A$1:$BC$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master_Data'!$A$1:$BB$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Merge_Audit'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Statistics'!$A$1:$N$2</definedName>
   </definedNames>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC9"/>
+  <dimension ref="A1:BB9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -471,20 +471,19 @@
     <col width="14" customWidth="1" min="39" max="39"/>
     <col width="12" customWidth="1" min="40" max="40"/>
     <col width="13" customWidth="1" min="41" max="41"/>
-    <col width="17" customWidth="1" min="42" max="42"/>
-    <col width="28" customWidth="1" min="43" max="43"/>
-    <col width="12" customWidth="1" min="44" max="44"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
+    <col width="39" customWidth="1" min="44" max="44"/>
     <col width="12" customWidth="1" min="45" max="45"/>
-    <col width="12" customWidth="1" min="46" max="46"/>
-    <col width="21" customWidth="1" min="47" max="47"/>
-    <col width="25" customWidth="1" min="48" max="48"/>
-    <col width="23" customWidth="1" min="49" max="49"/>
+    <col width="21" customWidth="1" min="46" max="46"/>
+    <col width="25" customWidth="1" min="47" max="47"/>
+    <col width="23" customWidth="1" min="48" max="48"/>
+    <col width="12" customWidth="1" min="49" max="49"/>
     <col width="12" customWidth="1" min="50" max="50"/>
-    <col width="12" customWidth="1" min="51" max="51"/>
-    <col width="15" customWidth="1" min="52" max="52"/>
+    <col width="15" customWidth="1" min="51" max="51"/>
+    <col width="12" customWidth="1" min="52" max="52"/>
     <col width="12" customWidth="1" min="53" max="53"/>
-    <col width="12" customWidth="1" min="54" max="54"/>
-    <col width="14" customWidth="1" min="55" max="55"/>
+    <col width="14" customWidth="1" min="54" max="54"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -695,70 +694,65 @@
       </c>
       <c r="AP1" s="2" t="inlineStr">
         <is>
-          <t>Pack Size (MOQ)</t>
+          <t>Cust Group</t>
         </is>
       </c>
       <c r="AQ1" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve"> Cont ID </t>
+        </is>
+      </c>
+      <c r="AR1" s="2" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="AS1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Jul-26 </t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> July'26- Forecast </t>
+        </is>
+      </c>
+      <c r="AU1" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Avg Jan'26 to June'26 </t>
+        </is>
+      </c>
+      <c r="AV1" s="2" t="inlineStr">
+        <is>
+          <t>Customer buying group</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
+        <is>
+          <t>Award Type</t>
+        </is>
+      </c>
+      <c r="AX1" s="2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="AY1" s="2" t="inlineStr">
+        <is>
+          <t>Sold to party</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
+        <is>
           <t>Lookup</t>
         </is>
       </c>
-      <c r="AR1" s="2" t="inlineStr">
-        <is>
-          <t>Cust Group</t>
-        </is>
-      </c>
-      <c r="AS1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Cont ID </t>
-        </is>
-      </c>
-      <c r="AT1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Jul-26 </t>
-        </is>
-      </c>
-      <c r="AU1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> July'26- Forecast </t>
-        </is>
-      </c>
-      <c r="AV1" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> Avg Jan'26 to June'26 </t>
-        </is>
-      </c>
-      <c r="AW1" s="2" t="inlineStr">
-        <is>
-          <t>Customer buying group</t>
-        </is>
-      </c>
-      <c r="AX1" s="2" t="inlineStr">
-        <is>
-          <t>Award Type</t>
-        </is>
-      </c>
-      <c r="AY1" s="2" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="AZ1" s="2" t="inlineStr">
-        <is>
-          <t>Sold to party</t>
-        </is>
-      </c>
       <c r="BA1" s="2" t="inlineStr">
         <is>
-          <t>NDC</t>
+          <t>Comments</t>
         </is>
       </c>
       <c r="BB1" s="2" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-      <c r="BC1" s="2" t="inlineStr">
         <is>
           <t>Customer ETA</t>
         </is>
@@ -879,6 +873,36 @@
       <c r="AG2" s="3" t="n">
         <v>46240</v>
       </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>S2ECON</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>64380018701Auburn Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> -   </t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6 </t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8 </t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1014,37 +1038,34 @@
           <t>64380-201-01</t>
         </is>
       </c>
-      <c r="AP3" t="n">
-        <v>24</v>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>WBAD</t>
+        </is>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>64380020101EXPRESS SCRIPTS</t>
+          <t>ABCS0614</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>Econdisc</t>
+          <t>64380020101CENCORA GLOBAL PROCUREMENT</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>S2ECON</t>
+          <t xml:space="preserve"> 144 </t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 432 </t>
+          <t xml:space="preserve"> 250 </t>
         </is>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 366 </t>
-        </is>
-      </c>
-      <c r="AV3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 276 </t>
+          <t xml:space="preserve"> 220 </t>
         </is>
       </c>
     </row>
@@ -1163,6 +1184,36 @@
       <c r="AG4" s="3" t="n">
         <v>46240</v>
       </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>S2ECON</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>64380018701Auburn Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> -   </t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6 </t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8 </t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1298,37 +1349,34 @@
           <t>64380-201-01</t>
         </is>
       </c>
-      <c r="AP5" t="n">
-        <v>24</v>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>WBAD</t>
+        </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>64380020101EXPRESS SCRIPTS</t>
+          <t>ABCS0614</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>Econdisc</t>
+          <t>64380020101CENCORA GLOBAL PROCUREMENT</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>S2ECON</t>
+          <t xml:space="preserve"> 144 </t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 432 </t>
+          <t xml:space="preserve"> 250 </t>
         </is>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 366 </t>
-        </is>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 276 </t>
+          <t xml:space="preserve"> 220 </t>
         </is>
       </c>
     </row>
@@ -1447,6 +1495,36 @@
       <c r="AG6" s="3" t="n">
         <v>46240</v>
       </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>S2ECON</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>64380018701Auburn Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> -   </t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6 </t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8 </t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1582,37 +1660,34 @@
           <t>64380-201-01</t>
         </is>
       </c>
-      <c r="AP7" t="n">
-        <v>24</v>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>WBAD</t>
+        </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>64380020101EXPRESS SCRIPTS</t>
+          <t>ABCS0614</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>Econdisc</t>
+          <t>64380020101CENCORA GLOBAL PROCUREMENT</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>S2ECON</t>
+          <t xml:space="preserve"> 144 </t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 432 </t>
+          <t xml:space="preserve"> 250 </t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 366 </t>
-        </is>
-      </c>
-      <c r="AV7" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 276 </t>
+          <t xml:space="preserve"> 220 </t>
         </is>
       </c>
     </row>
@@ -1731,6 +1806,36 @@
       <c r="AG8" s="3" t="n">
         <v>46240</v>
       </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>S2ECON</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>64380018701Auburn Pharmaceuticals</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> -   </t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 6 </t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 8 </t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1866,42 +1971,39 @@
           <t>64380-201-01</t>
         </is>
       </c>
-      <c r="AP9" t="n">
-        <v>24</v>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>WBAD</t>
+        </is>
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>64380020101EXPRESS SCRIPTS</t>
+          <t>ABCS0614</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>Econdisc</t>
+          <t>64380020101CENCORA GLOBAL PROCUREMENT</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>S2ECON</t>
+          <t xml:space="preserve"> 144 </t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 432 </t>
+          <t xml:space="preserve"> 250 </t>
         </is>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 366 </t>
-        </is>
-      </c>
-      <c r="AV9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 276 </t>
+          <t xml:space="preserve"> 220 </t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BC9"/>
+  <autoFilter ref="A1:BB9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2050,18 +2152,8 @@
           <t>sales_summ.xlsx</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Pack Size (MOQ), Lookup</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>NDC Code</t>
-        </is>
-      </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -2071,7 +2163,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>NDC Code; conflicting values=0</t>
+          <t>Source dataframe missing or empty</t>
         </is>
       </c>
     </row>
@@ -2083,26 +2175,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cust Group,  Cont ID ,  Jul-26 ,  July'26- Forecast ,  Avg Jan'26 to June'26 </t>
+          <t xml:space="preserve">Cust Group,  Cont ID , x,  Jul-26 ,  July'26- Forecast ,  Avg Jan'26 to June'26 </t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Lookup</t>
+          <t>NDC Code</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lookup; conflicting values=0</t>
+          <t>NDC Code; conflicting values=24</t>
         </is>
       </c>
     </row>
@@ -2145,26 +2237,26 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Award Type, Customer, Sold to party, NDC</t>
+          <t>Award Type, Customer, Sold to party, Lookup</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Lookup</t>
+          <t>NDC Code</t>
         </is>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>129</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Lookup; conflicting values=0</t>
+          <t>NDC Code; conflicting values=11</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2414,7 @@
         <v>6</v>
       </c>
       <c r="G2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fixed buying groups issue
</commit_message>
<xml_diff>
--- a/OrderbookAutomation/output/Business_Master_Data.xlsx
+++ b/OrderbookAutomation/output/Business_Master_Data.xlsx
@@ -11,12 +11,14 @@
     <sheet name="Merge_Audit" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Statistics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Buying_Group_Exceptions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Buying_Group_Audit" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master_Data'!$A$1:$BC$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master_Data'!$A$1:$BE$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Merge_Audit'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Statistics'!$A$1:$N$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Buying_Group_Exceptions'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Buying_Group_Exceptions'!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Buying_Group_Audit'!$A$1:$B$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BC9"/>
+  <dimension ref="A1:BE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -486,7 +488,9 @@
     <col width="12" customWidth="1" min="52" max="52"/>
     <col width="14" customWidth="1" min="53" max="53"/>
     <col width="23" customWidth="1" min="54" max="54"/>
-    <col width="28" customWidth="1" min="55" max="55"/>
+    <col width="21" customWidth="1" min="55" max="55"/>
+    <col width="28" customWidth="1" min="56" max="56"/>
+    <col width="14" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -762,7 +766,17 @@
       </c>
       <c r="BC1" s="2" t="inlineStr">
         <is>
+          <t>Buying Group Source</t>
+        </is>
+      </c>
+      <c r="BD1" s="2" t="inlineStr">
+        <is>
           <t>Buying Group Lookup Status</t>
+        </is>
+      </c>
+      <c r="BE1" s="2" t="inlineStr">
+        <is>
+          <t>Buying Group</t>
         </is>
       </c>
     </row>
@@ -911,9 +925,24 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
@@ -1081,9 +1110,24 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC3" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
@@ -1232,9 +1276,24 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
@@ -1402,9 +1461,24 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
@@ -1553,9 +1627,24 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC6" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
@@ -1723,9 +1812,24 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
@@ -1874,9 +1978,24 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC8" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
@@ -2044,14 +2163,29 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC9" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BC9"/>
+  <autoFilter ref="A1:BE9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2065,7 +2199,7 @@
   <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -2311,7 +2445,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Buying_groups.xlsx</t>
+          <t>Buying_groups.xlsx, Strend.xlsx, Open_Order_Summary.xlsx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2325,17 +2459,17 @@
         </is>
       </c>
       <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
         <v>0</v>
-      </c>
-      <c r="E9" t="n">
-        <v>8</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Dedicated Buying Group lookup; exact_duplicate_source_rows_removed=666; conflicting_customers=0</t>
+          <t>Multi-source Buying Group lookup (priority-resolved); exact_duplicate_source_rows_removed=717; same_priority_conflicts=0; lower_priority_disagreements=2; matches_by_source={'Strend.xlsx': 8}</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2608,7 @@
         <v>4</v>
       </c>
       <c r="K2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
         <v>8</v>
@@ -2498,14 +2632,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2521,15 +2658,30 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Buying Group(s)</t>
+          <t>Selected Buying Group</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Rejected Buying Group</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Selected Source</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Rejected Source</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
@@ -2538,27 +2690,312 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>CENCORA GLOBAL PROCUREMENT</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KROGER</t>
+          <t>CENCORA GLOBAL PROCUREMENT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>WBAD</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NOT_FOUND</t>
+          <t>ABC</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Customer not present in Buying Groups source workbook</t>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Open_Order_Summary.xlsx</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>LOWER_PRIORITY_DISAGREEMENT</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Resolved deterministically by source priority: Strend.xlsx (priority 2) outranks Open_Order_Summary.xlsx (priority 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mckesson Financial Center</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MCKESSON FINANCIAL CENTER</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ClarusOne</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>McKesson</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Open_Order_Summary.xlsx</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>LOWER_PRIORITY_DISAGREEMENT</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Resolved deterministically by source priority: Strend.xlsx (priority 2) outranks Open_Order_Summary.xlsx (priority 3)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:H3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Total master rows</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Master rows after merge</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unique master customers</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Unique consolidated source customers</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Exact duplicate source rows removed</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Matched rows</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NOT_FOUND rows</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DUPLICATE_CONFLICT rows</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Same-priority conflicting customers</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lower-priority disagreements</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Populated Buying Group rows</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Blank Buying Group rows</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Source record count - Buying_groups.xlsx (priority 1)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Master rows matched from Buying_groups.xlsx</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Source record count - Strend.xlsx (priority 2)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Master rows matched from Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Source record count - Open_Order_Summary.xlsx (priority 3)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Master rows matched from Open_Order_Summary.xlsx</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Final source for customer 'KROGER'</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Strend.xlsx -&gt; Econdisc</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
final data bug fixes
</commit_message>
<xml_diff>
--- a/OrderbookAutomation/output/Business_Master_Data.xlsx
+++ b/OrderbookAutomation/output/Business_Master_Data.xlsx
@@ -12,13 +12,15 @@
     <sheet name="Statistics" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Buying_Group_Exceptions" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Buying_Group_Audit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Award_Exceptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master_Data'!$A$1:$BE$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master_Data'!$A$1:$BD$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Merge_Audit'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Statistics'!$A$1:$N$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Buying_Group_Exceptions'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Buying_Group_Audit'!$A$1:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Award_Exceptions'!$A$1:$G$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE9"/>
+  <dimension ref="A1:BD9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -482,15 +484,14 @@
     <col width="21" customWidth="1" min="46" max="46"/>
     <col width="25" customWidth="1" min="47" max="47"/>
     <col width="12" customWidth="1" min="48" max="48"/>
-    <col width="12" customWidth="1" min="49" max="49"/>
-    <col width="15" customWidth="1" min="50" max="50"/>
-    <col width="12" customWidth="1" min="51" max="51"/>
-    <col width="12" customWidth="1" min="52" max="52"/>
+    <col width="14" customWidth="1" min="49" max="49"/>
+    <col width="23" customWidth="1" min="50" max="50"/>
+    <col width="21" customWidth="1" min="51" max="51"/>
+    <col width="28" customWidth="1" min="52" max="52"/>
     <col width="14" customWidth="1" min="53" max="53"/>
-    <col width="23" customWidth="1" min="54" max="54"/>
+    <col width="12" customWidth="1" min="54" max="54"/>
     <col width="21" customWidth="1" min="55" max="55"/>
-    <col width="28" customWidth="1" min="56" max="56"/>
-    <col width="14" customWidth="1" min="57" max="57"/>
+    <col width="22" customWidth="1" min="56" max="56"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -731,52 +732,47 @@
       </c>
       <c r="AV1" s="2" t="inlineStr">
         <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
+        <is>
+          <t>Customer ETA</t>
+        </is>
+      </c>
+      <c r="AX1" s="2" t="inlineStr">
+        <is>
+          <t>Customer buying group</t>
+        </is>
+      </c>
+      <c r="AY1" s="2" t="inlineStr">
+        <is>
+          <t>Buying Group Source</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
+        <is>
+          <t>Buying Group Lookup Status</t>
+        </is>
+      </c>
+      <c r="BA1" s="2" t="inlineStr">
+        <is>
+          <t>Buying Group</t>
+        </is>
+      </c>
+      <c r="BB1" s="2" t="inlineStr">
+        <is>
           <t>Award Type</t>
         </is>
       </c>
-      <c r="AW1" s="2" t="inlineStr">
-        <is>
-          <t>Customer</t>
-        </is>
-      </c>
-      <c r="AX1" s="2" t="inlineStr">
-        <is>
-          <t>Sold to party</t>
-        </is>
-      </c>
-      <c r="AY1" s="2" t="inlineStr">
-        <is>
-          <t>NDC</t>
-        </is>
-      </c>
-      <c r="AZ1" s="2" t="inlineStr">
-        <is>
-          <t>Comments</t>
-        </is>
-      </c>
-      <c r="BA1" s="2" t="inlineStr">
-        <is>
-          <t>Customer ETA</t>
-        </is>
-      </c>
-      <c r="BB1" s="2" t="inlineStr">
-        <is>
-          <t>Customer buying group</t>
-        </is>
-      </c>
       <c r="BC1" s="2" t="inlineStr">
         <is>
-          <t>Buying Group Source</t>
+          <t>Award Lookup Status</t>
         </is>
       </c>
       <c r="BD1" s="2" t="inlineStr">
         <is>
-          <t>Buying Group Lookup Status</t>
-        </is>
-      </c>
-      <c r="BE1" s="2" t="inlineStr">
-        <is>
-          <t>Buying Group</t>
+          <t>Award Match Strategy</t>
         </is>
       </c>
     </row>
@@ -925,24 +921,29 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
-      <c r="BB2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
@@ -1110,24 +1111,29 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
-      <c r="BB3" t="inlineStr">
+      <c r="AX3" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC3" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE3" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
@@ -1276,24 +1282,29 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
-      <c r="BB4" t="inlineStr">
+      <c r="AX4" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD4" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE4" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
@@ -1461,24 +1472,29 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
-      <c r="BB5" t="inlineStr">
+      <c r="AX5" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD5" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE5" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
@@ -1627,24 +1643,29 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
-      <c r="BB6" t="inlineStr">
+      <c r="AX6" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC6" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD6" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE6" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
@@ -1812,24 +1833,29 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
-      <c r="BB7" t="inlineStr">
+      <c r="AX7" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD7" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE7" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
@@ -1978,24 +2004,29 @@
           <t xml:space="preserve"> 132 </t>
         </is>
       </c>
-      <c r="BB8" t="inlineStr">
+      <c r="AX8" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC8" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD8" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE8" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
@@ -2163,29 +2194,34 @@
           <t xml:space="preserve"> 324 </t>
         </is>
       </c>
-      <c r="BB9" t="inlineStr">
+      <c r="AX9" t="inlineStr">
         <is>
           <t>Econdisc</t>
         </is>
       </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>Strend.xlsx</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>MATCHED</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>Econdisc</t>
+        </is>
+      </c>
       <c r="BC9" t="inlineStr">
         <is>
-          <t>Strend.xlsx</t>
-        </is>
-      </c>
-      <c r="BD9" t="inlineStr">
-        <is>
-          <t>MATCHED</t>
-        </is>
-      </c>
-      <c r="BE9" t="inlineStr">
-        <is>
-          <t>Econdisc</t>
+          <t>NOT_FOUND</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BE9"/>
+  <autoFilter ref="A1:BD9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2201,7 +2237,7 @@
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -2383,93 +2419,93 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Awards.xlsx</t>
+          <t>CIP.xlsx</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Award Type, Customer, Sold to party, NDC</t>
+          <t>Comments, Customer ETA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Lookup</t>
+          <t>NDC Code</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>129</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lookup; conflicting values=0</t>
+          <t>NDC Code; conflicting values=0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CIP.xlsx</t>
+          <t>Buying_groups.xlsx, Strend.xlsx, Open_Order_Summary.xlsx</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Comments, Customer ETA</t>
+          <t>Customer buying group</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>NDC Code</t>
+          <t>Sold-to party Name</t>
         </is>
       </c>
       <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
         <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>10</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>NDC Code; conflicting values=0</t>
+          <t>Multi-source Buying Group lookup (priority-resolved); exact_duplicate_source_rows_removed=717; same_priority_conflicts=0; lower_priority_disagreements=2; matches_by_source={'Strend.xlsx': 8}</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Buying_groups.xlsx, Strend.xlsx, Open_Order_Summary.xlsx</t>
+          <t>Awards.xlsx</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Customer buying group</t>
+          <t>Award Type</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sold-to party Name</t>
+          <t>Lookup (Customer+NDC), NDC Code fallback</t>
         </is>
       </c>
       <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>8</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Multi-source Buying Group lookup (priority-resolved); exact_duplicate_source_rows_removed=717; same_priority_conflicts=0; lower_priority_disagreements=2; matches_by_source={'Strend.xlsx': 8}</t>
+          <t>Dedicated Award lookup at Customer+NDC grain; matched_by_lookup=0; matched_by_ndc=0; not_found=8; duplicate_conflict=0</t>
         </is>
       </c>
     </row>
@@ -2998,4 +3034,169 @@
   <autoFilter ref="A1:B20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Customer</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>NDC</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Lookup</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Award Type</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Match Strategy</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>64380016101</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Backup (Primary CVS); No Award; No award; Primary</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>NDC (product-level fallback)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>DUPLICATE_CONFLICT</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>NDC maps to multiple distinct Award Type values across customers; ambiguous at product level</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>64380072701</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Backup; No Award; Primary</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NDC (product-level fallback)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>DUPLICATE_CONFLICT</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>NDC maps to multiple distinct Award Type values across customers; ambiguous at product level</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>KROGER</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>64380018701</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>64380018701KROGER</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>No Award record found by Lookup (Customer+NDC) or by NDC in the Awards source</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KROGER</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64380020101</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>64380020101KROGER</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>No Award record found by Lookup (Customer+NDC) or by NDC in the Awards source</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>